<commit_message>
remove no longer used IO files, fix units for WMITR
</commit_message>
<xml_diff>
--- a/InputData/io-model/WMITR/Worker Marg Income Tax Rate.xlsx
+++ b/InputData/io-model/WMITR/Worker Marg Income Tax Rate.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28627"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29530"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Meghan\Dropbox (Energy Innovation)\EPS Versions\eps-1.5.0-us-wipL\InputData\indst\WMITR\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Olivia Ashmoore\Documents\EPS_Models by Region\eps-mexico\InputData\io-model\WMITR\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="126" documentId="11_5D3CDC222100BEE762BE85B664AA361E9EA1AC7E" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{86E733F2-E4EE-4B9D-B0DA-79970A75C6D1}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86E1F14D-41AB-4E47-8CFE-404AB65BF76F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="120" yWindow="105" windowWidth="25875" windowHeight="11055" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -18,9 +18,6 @@
     <sheet name="Calculations" sheetId="4" r:id="rId3"/>
     <sheet name="WMITR" sheetId="2" r:id="rId4"/>
   </sheets>
-  <externalReferences>
-    <externalReference r:id="rId5"/>
-  </externalReferences>
   <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -186,7 +183,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.000"/>
   </numFmts>
-  <fonts count="14">
+  <fonts count="14" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -245,32 +242,38 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="7">
@@ -454,65 +457,53 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="10" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="10" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="3" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="10" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="3" fontId="4" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="3" fontId="7" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="3" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="9" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="10" fontId="4" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="10" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="7" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="9" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="10" fontId="4" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1" readingOrder="1"/>
@@ -526,12 +517,19 @@
     <xf numFmtId="0" fontId="13" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="4" fontId="9" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="4" fontId="9" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment readingOrder="1"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -548,19 +546,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <sheetNames>
-      <sheetName val="About"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -850,313 +835,311 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J36"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <dimension ref="A1:J34"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.28515625" customWidth="1"/>
     <col min="2" max="2" width="27.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="15">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="4"/>
-      <c r="C1" s="5"/>
-      <c r="D1" s="5"/>
-      <c r="E1" s="5"/>
-    </row>
-    <row r="2" spans="1:10" ht="15">
-      <c r="A2" s="5"/>
-      <c r="B2" s="5"/>
-      <c r="C2" s="5"/>
-      <c r="D2" s="5"/>
-      <c r="E2" s="5"/>
-    </row>
-    <row r="3" spans="1:10" ht="15">
+      <c r="B1" s="3"/>
+      <c r="C1" s="4"/>
+      <c r="D1" s="4"/>
+      <c r="E1" s="4"/>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A2" s="4"/>
+      <c r="B2" s="4"/>
+      <c r="C2" s="4"/>
+      <c r="D2" s="4"/>
+      <c r="E2" s="4"/>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="D3" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="E3" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="J3" s="35" t="s">
+      <c r="C3" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="J3" s="30" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="15">
-      <c r="A4" s="5"/>
-      <c r="B4" s="5" t="s">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A4" s="4"/>
+      <c r="B4" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="5"/>
-      <c r="D4" s="5"/>
-      <c r="E4" s="5"/>
-      <c r="J4" s="41" t="s">
+      <c r="C4" s="4"/>
+      <c r="D4" s="4"/>
+      <c r="E4" s="4"/>
+      <c r="J4" s="35" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="15">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="3"/>
-      <c r="B5" s="5">
+      <c r="B5" s="4">
         <v>2019</v>
       </c>
-      <c r="C5" s="5"/>
-      <c r="D5" s="5"/>
-      <c r="E5" s="5"/>
-      <c r="J5" s="42" t="s">
+      <c r="C5" s="4"/>
+      <c r="D5" s="4"/>
+      <c r="E5" s="4"/>
+      <c r="J5" s="36" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ht="15">
-      <c r="A6" s="5"/>
-      <c r="B6" s="5" t="s">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A6" s="4"/>
+      <c r="B6" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="C6" s="7"/>
-      <c r="D6" s="7"/>
-      <c r="E6" s="5"/>
-      <c r="J6" s="42" t="s">
+      <c r="C6" s="4"/>
+      <c r="D6" s="4"/>
+      <c r="E6" s="4"/>
+      <c r="J6" s="36" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="15">
-      <c r="A7" s="5"/>
-      <c r="B7" s="8" t="s">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A7" s="4"/>
+      <c r="B7" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="C7" s="9"/>
-      <c r="D7" s="9"/>
-      <c r="E7" s="9"/>
-      <c r="J7" s="42" t="s">
+      <c r="C7" s="7"/>
+      <c r="D7" s="7"/>
+      <c r="E7" s="7"/>
+      <c r="J7" s="36" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="8" spans="1:10" ht="15">
-      <c r="A8" s="5"/>
-      <c r="B8" s="5"/>
-      <c r="C8" s="5"/>
-      <c r="D8" s="5"/>
-      <c r="E8" s="5"/>
-    </row>
-    <row r="9" spans="1:10" ht="15">
-      <c r="A9" s="5"/>
-      <c r="B9" s="5" t="s">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A8" s="4"/>
+      <c r="B8" s="4"/>
+      <c r="C8" s="4"/>
+      <c r="D8" s="4"/>
+      <c r="E8" s="4"/>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A9" s="4"/>
+      <c r="B9" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="C9" s="5"/>
-      <c r="D9" s="5"/>
-      <c r="E9" s="5"/>
-    </row>
-    <row r="10" spans="1:10" ht="15">
-      <c r="A10" s="5"/>
-      <c r="B10" s="5">
+      <c r="C9" s="4"/>
+      <c r="D9" s="4"/>
+      <c r="E9" s="4"/>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A10" s="4"/>
+      <c r="B10" s="4">
         <v>2019</v>
       </c>
-      <c r="C10" s="5"/>
-      <c r="D10" s="5"/>
-      <c r="E10" s="5"/>
-    </row>
-    <row r="11" spans="1:10" ht="15">
-      <c r="A11" s="5"/>
-      <c r="B11" s="5" t="s">
+      <c r="C10" s="4"/>
+      <c r="D10" s="4"/>
+      <c r="E10" s="4"/>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A11" s="4"/>
+      <c r="B11" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="C11" s="5"/>
-      <c r="D11" s="5"/>
-      <c r="E11" s="5"/>
-    </row>
-    <row r="12" spans="1:10" ht="15">
-      <c r="A12" s="5"/>
-      <c r="B12" s="10" t="s">
+      <c r="C11" s="4"/>
+      <c r="D11" s="4"/>
+      <c r="E11" s="4"/>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A12" s="4"/>
+      <c r="B12" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="C12" s="5"/>
-      <c r="D12" s="5"/>
-      <c r="E12" s="5"/>
-    </row>
-    <row r="13" spans="1:10" ht="15">
-      <c r="A13" s="5"/>
-      <c r="B13" s="5" t="s">
+      <c r="C12" s="4"/>
+      <c r="D12" s="4"/>
+      <c r="E12" s="4"/>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A13" s="4"/>
+      <c r="B13" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="C13" s="7"/>
-      <c r="D13" s="7"/>
-      <c r="E13" s="7"/>
-    </row>
-    <row r="14" spans="1:10" ht="15">
-      <c r="A14" s="5"/>
-      <c r="B14" s="5"/>
-      <c r="C14" s="5"/>
-      <c r="D14" s="5"/>
-      <c r="E14" s="5"/>
-    </row>
-    <row r="15" spans="1:10" ht="15">
-      <c r="A15" s="5"/>
-      <c r="B15" s="5"/>
-      <c r="C15" s="5"/>
-      <c r="D15" s="5"/>
-      <c r="E15" s="5"/>
-    </row>
-    <row r="16" spans="1:10" ht="15">
-      <c r="A16" s="5"/>
-      <c r="B16" s="6" t="s">
+      <c r="C13" s="4"/>
+      <c r="D13" s="4"/>
+      <c r="E13" s="4"/>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A14" s="4"/>
+      <c r="B14" s="4"/>
+      <c r="C14" s="4"/>
+      <c r="D14" s="4"/>
+      <c r="E14" s="4"/>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A15" s="4"/>
+      <c r="B15" s="4"/>
+      <c r="C15" s="4"/>
+      <c r="D15" s="4"/>
+      <c r="E15" s="4"/>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A16" s="4"/>
+      <c r="B16" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="C16" s="11"/>
-      <c r="D16" s="12" t="s">
-        <v>3</v>
-      </c>
-      <c r="E16" s="12" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" ht="15">
-      <c r="A17" s="5"/>
+      <c r="C16" s="5"/>
+      <c r="D16" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="E16" s="9" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A17" s="4"/>
       <c r="B17" t="s">
         <v>17</v>
       </c>
-      <c r="C17" s="5"/>
-      <c r="D17" s="5"/>
-      <c r="E17" s="5"/>
-      <c r="G17" s="41"/>
-    </row>
-    <row r="18" spans="1:7" ht="15">
-      <c r="A18" s="5"/>
-      <c r="B18" s="8" t="s">
+      <c r="C17" s="4"/>
+      <c r="D17" s="4"/>
+      <c r="E17" s="4"/>
+      <c r="G17" s="35"/>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A18" s="4"/>
+      <c r="B18" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="C18" s="5"/>
-      <c r="D18" s="5"/>
-      <c r="E18" s="5"/>
-      <c r="G18" s="42"/>
-    </row>
-    <row r="19" spans="1:7" ht="15">
-      <c r="A19" s="5"/>
-      <c r="B19" s="42" t="s">
+      <c r="C18" s="4"/>
+      <c r="D18" s="4"/>
+      <c r="E18" s="4"/>
+      <c r="G18" s="36"/>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A19" s="4"/>
+      <c r="B19" s="36" t="s">
         <v>7</v>
       </c>
-      <c r="C19" s="7"/>
-      <c r="D19" s="7"/>
-      <c r="E19" s="7"/>
-      <c r="G19" s="42"/>
-    </row>
-    <row r="20" spans="1:7" ht="15">
-      <c r="A20" s="5"/>
-      <c r="B20" s="42" t="s">
+      <c r="C19" s="4"/>
+      <c r="D19" s="4"/>
+      <c r="E19" s="4"/>
+      <c r="G19" s="36"/>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A20" s="4"/>
+      <c r="B20" s="36" t="s">
         <v>9</v>
       </c>
-      <c r="C20" s="9"/>
-      <c r="D20" s="9"/>
-      <c r="E20" s="9"/>
-      <c r="G20" s="42"/>
-    </row>
-    <row r="21" spans="1:7" ht="15">
-      <c r="A21" s="5"/>
-      <c r="B21" s="42" t="s">
+      <c r="C20" s="7"/>
+      <c r="D20" s="7"/>
+      <c r="E20" s="7"/>
+      <c r="G20" s="36"/>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A21" s="4"/>
+      <c r="B21" s="36" t="s">
         <v>11</v>
       </c>
-      <c r="C21" s="5"/>
-      <c r="D21" s="5"/>
-      <c r="E21" s="5"/>
-    </row>
-    <row r="22" spans="1:7" customFormat="1" ht="15">
-      <c r="A22" s="5"/>
+      <c r="C21" s="4"/>
+      <c r="D21" s="4"/>
+      <c r="E21" s="4"/>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A22" s="4"/>
       <c r="B22" t="s">
         <v>18</v>
       </c>
-      <c r="C22" s="5"/>
-      <c r="D22" s="5"/>
-      <c r="E22" s="5"/>
-    </row>
-    <row r="23" spans="1:7" customFormat="1" ht="15">
-      <c r="A23" s="5"/>
-      <c r="C23" s="5"/>
-      <c r="D23" s="5"/>
-      <c r="E23" s="5"/>
-    </row>
-    <row r="24" spans="1:7" s="42" customFormat="1" ht="15"/>
-    <row r="25" spans="1:7" s="42" customFormat="1" ht="15"/>
-    <row r="26" spans="1:7" s="42" customFormat="1" ht="15"/>
-    <row r="27" spans="1:7" customFormat="1" ht="15">
-      <c r="A27" s="5"/>
-      <c r="B27" s="5"/>
-      <c r="C27" s="5"/>
-      <c r="D27" s="5"/>
-      <c r="E27" s="5"/>
-    </row>
-    <row r="28" spans="1:7" customFormat="1" ht="15">
+      <c r="C22" s="4"/>
+      <c r="D22" s="4"/>
+      <c r="E22" s="4"/>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A23" s="4"/>
+      <c r="C23" s="4"/>
+      <c r="D23" s="4"/>
+      <c r="E23" s="4"/>
+    </row>
+    <row r="24" spans="1:7" s="36" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="25" spans="1:7" s="36" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="26" spans="1:7" s="36" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A27" s="4"/>
+      <c r="B27" s="4"/>
+      <c r="C27" s="4"/>
+      <c r="D27" s="4"/>
+      <c r="E27" s="4"/>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="B28" s="5"/>
-      <c r="C28" s="36"/>
-      <c r="D28" s="5"/>
-      <c r="E28" s="5"/>
-    </row>
-    <row r="29" spans="1:7" customFormat="1" ht="15">
-      <c r="A29" s="5" t="s">
+      <c r="B28" s="4"/>
+      <c r="C28" s="31"/>
+      <c r="D28" s="4"/>
+      <c r="E28" s="4"/>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A29" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="B29" s="36">
+      <c r="B29" s="31">
         <v>0.88711067149387013</v>
       </c>
-      <c r="C29" s="5"/>
-      <c r="D29" s="5"/>
-      <c r="E29" s="5"/>
-    </row>
-    <row r="30" spans="1:7" customFormat="1" ht="15">
-      <c r="A30" s="5"/>
-      <c r="B30" s="5"/>
-      <c r="C30" s="8"/>
-      <c r="D30" s="9"/>
-      <c r="E30" s="9"/>
-    </row>
-    <row r="31" spans="1:7" customFormat="1" ht="15">
+      <c r="C29" s="4"/>
+      <c r="D29" s="4"/>
+      <c r="E29" s="4"/>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A30" s="4"/>
+      <c r="B30" s="4"/>
+      <c r="C30" s="6"/>
+      <c r="D30" s="7"/>
+      <c r="E30" s="7"/>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="B31" s="5"/>
-      <c r="C31" s="5" t="s">
+      <c r="B31" s="4"/>
+      <c r="C31" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="D31" s="5"/>
-      <c r="E31" s="5"/>
-    </row>
-    <row r="32" spans="1:7" customFormat="1" ht="15">
-      <c r="A32" s="5">
+      <c r="D31" s="4"/>
+      <c r="E31" s="4"/>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A32" s="4">
         <v>2012</v>
       </c>
-      <c r="B32" s="5">
+      <c r="B32" s="4">
         <v>19.95</v>
       </c>
-      <c r="C32" s="5"/>
-      <c r="D32" s="5"/>
-      <c r="E32" s="5"/>
-    </row>
-    <row r="33" spans="3:5" customFormat="1" ht="15">
-      <c r="C33" s="5"/>
-      <c r="D33" s="5"/>
-      <c r="E33" s="5"/>
-    </row>
-    <row r="34" spans="3:5" customFormat="1" ht="15">
-      <c r="C34" s="5" t="s">
+      <c r="C32" s="4"/>
+      <c r="D32" s="4"/>
+      <c r="E32" s="4"/>
+    </row>
+    <row r="33" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C33" s="4"/>
+      <c r="D33" s="4"/>
+      <c r="E33" s="4"/>
+    </row>
+    <row r="34" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C34" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="D34" s="7"/>
-      <c r="E34" s="7"/>
-    </row>
-    <row r="35" spans="3:5" customFormat="1" ht="15"/>
-    <row r="36" spans="3:5" customFormat="1" ht="15"/>
+      <c r="D34" s="4"/>
+      <c r="E34" s="4"/>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="B7" r:id="rId1" xr:uid="{8A0F0CE5-0BE2-487A-97D0-20F5BE6BE8FD}"/>
@@ -1171,257 +1154,255 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1BAE8291-937B-4F44-8511-6E1543869991}">
   <dimension ref="A1:AT12"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="9.140625" style="37"/>
-    <col min="3" max="3" width="20.85546875" style="37" customWidth="1"/>
-    <col min="4" max="16384" width="9.140625" style="37"/>
+    <col min="3" max="3" width="20.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:46">
-      <c r="A1" s="41" t="s">
+    <row r="1" spans="1:46" x14ac:dyDescent="0.25">
+      <c r="A1" s="35" t="s">
         <v>6</v>
       </c>
-      <c r="B1" s="5"/>
-      <c r="C1" s="5"/>
-      <c r="D1" s="5"/>
-      <c r="E1" s="38"/>
-      <c r="G1" s="38"/>
-      <c r="H1" s="38"/>
-      <c r="I1" s="38"/>
-      <c r="J1" s="38"/>
-      <c r="K1" s="38"/>
-      <c r="L1" s="38"/>
-      <c r="M1" s="38"/>
-      <c r="N1" s="38"/>
-      <c r="Q1" s="38"/>
-      <c r="R1" s="38"/>
-      <c r="S1" s="38"/>
-      <c r="T1" s="38"/>
-      <c r="U1" s="38"/>
-      <c r="V1" s="38"/>
-      <c r="W1" s="38"/>
-      <c r="Y1" s="38"/>
-      <c r="Z1" s="38"/>
-      <c r="AA1" s="38"/>
-      <c r="AB1" s="38"/>
-      <c r="AC1" s="38"/>
-      <c r="AD1" s="38"/>
-      <c r="AE1" s="38"/>
-      <c r="AF1" s="38"/>
-      <c r="AG1" s="38"/>
-      <c r="AH1" s="38"/>
-      <c r="AI1" s="38"/>
-      <c r="AJ1" s="38"/>
-      <c r="AK1" s="38"/>
-      <c r="AL1" s="38"/>
-      <c r="AM1" s="38"/>
-      <c r="AN1" s="38"/>
-      <c r="AO1" s="38"/>
-      <c r="AP1" s="38"/>
-      <c r="AQ1" s="38"/>
-      <c r="AR1" s="38"/>
-      <c r="AT1" s="38"/>
-    </row>
-    <row r="2" spans="1:46">
-      <c r="A2" s="42" t="s">
+      <c r="B1" s="4"/>
+      <c r="C1" s="4"/>
+      <c r="D1" s="4"/>
+      <c r="E1" s="32"/>
+      <c r="G1" s="32"/>
+      <c r="H1" s="32"/>
+      <c r="I1" s="32"/>
+      <c r="J1" s="32"/>
+      <c r="K1" s="32"/>
+      <c r="L1" s="32"/>
+      <c r="M1" s="32"/>
+      <c r="N1" s="32"/>
+      <c r="Q1" s="32"/>
+      <c r="R1" s="32"/>
+      <c r="S1" s="32"/>
+      <c r="T1" s="32"/>
+      <c r="U1" s="32"/>
+      <c r="V1" s="32"/>
+      <c r="W1" s="32"/>
+      <c r="Y1" s="32"/>
+      <c r="Z1" s="32"/>
+      <c r="AA1" s="32"/>
+      <c r="AB1" s="32"/>
+      <c r="AC1" s="32"/>
+      <c r="AD1" s="32"/>
+      <c r="AE1" s="32"/>
+      <c r="AF1" s="32"/>
+      <c r="AG1" s="32"/>
+      <c r="AH1" s="32"/>
+      <c r="AI1" s="32"/>
+      <c r="AJ1" s="32"/>
+      <c r="AK1" s="32"/>
+      <c r="AL1" s="32"/>
+      <c r="AM1" s="32"/>
+      <c r="AN1" s="32"/>
+      <c r="AO1" s="32"/>
+      <c r="AP1" s="32"/>
+      <c r="AQ1" s="32"/>
+      <c r="AR1" s="32"/>
+      <c r="AT1" s="32"/>
+    </row>
+    <row r="2" spans="1:46" x14ac:dyDescent="0.25">
+      <c r="A2" s="36" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="5"/>
-      <c r="C2" s="5"/>
-      <c r="D2" s="5"/>
-      <c r="E2" s="39"/>
-      <c r="F2" s="39"/>
-      <c r="G2" s="39"/>
-      <c r="H2" s="39"/>
-      <c r="I2" s="39"/>
-      <c r="J2" s="39"/>
-      <c r="K2" s="39"/>
-      <c r="L2" s="39"/>
-      <c r="M2" s="39"/>
-      <c r="N2" s="39"/>
-      <c r="O2" s="39"/>
-      <c r="P2" s="39"/>
-      <c r="Q2" s="39"/>
-      <c r="R2" s="39"/>
-      <c r="S2" s="39"/>
-      <c r="T2" s="39"/>
-      <c r="U2" s="39"/>
-      <c r="V2" s="39"/>
-      <c r="W2" s="39"/>
-      <c r="X2" s="39"/>
-      <c r="Y2" s="39"/>
-      <c r="Z2" s="39"/>
-      <c r="AA2" s="39"/>
-      <c r="AB2" s="39"/>
-      <c r="AC2" s="39"/>
-      <c r="AD2" s="39"/>
-      <c r="AE2" s="39"/>
-      <c r="AF2" s="39"/>
-      <c r="AG2" s="39"/>
-      <c r="AH2" s="39"/>
-      <c r="AI2" s="39"/>
-      <c r="AJ2" s="39"/>
-      <c r="AK2" s="39"/>
-      <c r="AL2" s="39"/>
-      <c r="AM2" s="39"/>
-      <c r="AN2" s="39"/>
-      <c r="AO2" s="39"/>
-      <c r="AP2" s="39"/>
-      <c r="AQ2" s="39"/>
-      <c r="AR2" s="39"/>
-      <c r="AS2" s="39"/>
-      <c r="AT2" s="39"/>
-    </row>
-    <row r="3" spans="1:46">
-      <c r="A3" s="42" t="s">
+      <c r="B2" s="4"/>
+      <c r="C2" s="4"/>
+      <c r="D2" s="4"/>
+      <c r="E2" s="33"/>
+      <c r="F2" s="33"/>
+      <c r="G2" s="33"/>
+      <c r="H2" s="33"/>
+      <c r="I2" s="33"/>
+      <c r="J2" s="33"/>
+      <c r="K2" s="33"/>
+      <c r="L2" s="33"/>
+      <c r="M2" s="33"/>
+      <c r="N2" s="33"/>
+      <c r="O2" s="33"/>
+      <c r="P2" s="33"/>
+      <c r="Q2" s="33"/>
+      <c r="R2" s="33"/>
+      <c r="S2" s="33"/>
+      <c r="T2" s="33"/>
+      <c r="U2" s="33"/>
+      <c r="V2" s="33"/>
+      <c r="W2" s="33"/>
+      <c r="X2" s="33"/>
+      <c r="Y2" s="33"/>
+      <c r="Z2" s="33"/>
+      <c r="AA2" s="33"/>
+      <c r="AB2" s="33"/>
+      <c r="AC2" s="33"/>
+      <c r="AD2" s="33"/>
+      <c r="AE2" s="33"/>
+      <c r="AF2" s="33"/>
+      <c r="AG2" s="33"/>
+      <c r="AH2" s="33"/>
+      <c r="AI2" s="33"/>
+      <c r="AJ2" s="33"/>
+      <c r="AK2" s="33"/>
+      <c r="AL2" s="33"/>
+      <c r="AM2" s="33"/>
+      <c r="AN2" s="33"/>
+      <c r="AO2" s="33"/>
+      <c r="AP2" s="33"/>
+      <c r="AQ2" s="33"/>
+      <c r="AR2" s="33"/>
+      <c r="AS2" s="33"/>
+      <c r="AT2" s="33"/>
+    </row>
+    <row r="3" spans="1:46" x14ac:dyDescent="0.25">
+      <c r="A3" s="36" t="s">
         <v>9</v>
       </c>
-      <c r="B3" s="5"/>
-      <c r="C3" s="5"/>
-      <c r="D3" s="5"/>
-      <c r="E3" s="39"/>
-      <c r="F3" s="39"/>
-      <c r="G3" s="39"/>
-      <c r="H3" s="39"/>
-      <c r="I3" s="39"/>
-      <c r="J3" s="39"/>
-      <c r="K3" s="39"/>
-      <c r="L3" s="39"/>
-      <c r="M3" s="39"/>
-      <c r="N3" s="39"/>
-      <c r="O3" s="39"/>
-      <c r="P3" s="39"/>
-      <c r="Q3" s="39"/>
-      <c r="R3" s="39"/>
-      <c r="S3" s="39"/>
-      <c r="T3" s="39"/>
-      <c r="U3" s="39"/>
-      <c r="V3" s="39"/>
-      <c r="W3" s="39"/>
-      <c r="X3" s="39"/>
-      <c r="Y3" s="39"/>
-      <c r="Z3" s="39"/>
-      <c r="AA3" s="39"/>
-      <c r="AB3" s="39"/>
-      <c r="AC3" s="39"/>
-      <c r="AD3" s="39"/>
-      <c r="AE3" s="39"/>
-      <c r="AF3" s="39"/>
-      <c r="AG3" s="39"/>
-      <c r="AH3" s="39"/>
-      <c r="AI3" s="39"/>
-      <c r="AJ3" s="39"/>
-      <c r="AK3" s="39"/>
-      <c r="AL3" s="39"/>
-      <c r="AM3" s="39"/>
-      <c r="AN3" s="39"/>
-      <c r="AO3" s="39"/>
-      <c r="AP3" s="39"/>
-      <c r="AQ3" s="39"/>
-      <c r="AR3" s="39"/>
-      <c r="AS3" s="39"/>
-      <c r="AT3" s="39"/>
-    </row>
-    <row r="4" spans="1:46">
-      <c r="A4" s="42" t="s">
+      <c r="B3" s="4"/>
+      <c r="C3" s="4"/>
+      <c r="D3" s="4"/>
+      <c r="E3" s="33"/>
+      <c r="F3" s="33"/>
+      <c r="G3" s="33"/>
+      <c r="H3" s="33"/>
+      <c r="I3" s="33"/>
+      <c r="J3" s="33"/>
+      <c r="K3" s="33"/>
+      <c r="L3" s="33"/>
+      <c r="M3" s="33"/>
+      <c r="N3" s="33"/>
+      <c r="O3" s="33"/>
+      <c r="P3" s="33"/>
+      <c r="Q3" s="33"/>
+      <c r="R3" s="33"/>
+      <c r="S3" s="33"/>
+      <c r="T3" s="33"/>
+      <c r="U3" s="33"/>
+      <c r="V3" s="33"/>
+      <c r="W3" s="33"/>
+      <c r="X3" s="33"/>
+      <c r="Y3" s="33"/>
+      <c r="Z3" s="33"/>
+      <c r="AA3" s="33"/>
+      <c r="AB3" s="33"/>
+      <c r="AC3" s="33"/>
+      <c r="AD3" s="33"/>
+      <c r="AE3" s="33"/>
+      <c r="AF3" s="33"/>
+      <c r="AG3" s="33"/>
+      <c r="AH3" s="33"/>
+      <c r="AI3" s="33"/>
+      <c r="AJ3" s="33"/>
+      <c r="AK3" s="33"/>
+      <c r="AL3" s="33"/>
+      <c r="AM3" s="33"/>
+      <c r="AN3" s="33"/>
+      <c r="AO3" s="33"/>
+      <c r="AP3" s="33"/>
+      <c r="AQ3" s="33"/>
+      <c r="AR3" s="33"/>
+      <c r="AS3" s="33"/>
+      <c r="AT3" s="33"/>
+    </row>
+    <row r="4" spans="1:46" x14ac:dyDescent="0.25">
+      <c r="A4" s="36" t="s">
         <v>11</v>
       </c>
-      <c r="B4" s="5"/>
-      <c r="C4" s="5"/>
-      <c r="D4" s="5"/>
-    </row>
-    <row r="5" spans="1:46">
-      <c r="A5" s="5"/>
-      <c r="B5" s="5"/>
-      <c r="C5" s="5"/>
-      <c r="D5" s="5"/>
-      <c r="E5" s="38"/>
-      <c r="O5" s="38"/>
-      <c r="P5" s="38"/>
-      <c r="X5" s="40"/>
-      <c r="Y5" s="38"/>
-    </row>
-    <row r="6" spans="1:46">
+      <c r="B4" s="4"/>
+      <c r="C4" s="4"/>
+      <c r="D4" s="4"/>
+    </row>
+    <row r="5" spans="1:46" x14ac:dyDescent="0.25">
+      <c r="A5" s="4"/>
+      <c r="B5" s="4"/>
+      <c r="C5" s="4"/>
+      <c r="D5" s="4"/>
+      <c r="E5" s="32"/>
+      <c r="O5" s="32"/>
+      <c r="P5" s="32"/>
+      <c r="X5" s="34"/>
+      <c r="Y5" s="32"/>
+    </row>
+    <row r="6" spans="1:46" x14ac:dyDescent="0.25">
       <c r="A6" s="43" t="s">
         <v>24</v>
       </c>
       <c r="B6" s="44"/>
-      <c r="C6" s="45" t="s">
+      <c r="C6" s="37" t="s">
         <v>25</v>
       </c>
-      <c r="D6" s="5"/>
-      <c r="O6" s="38"/>
-      <c r="P6" s="38"/>
-      <c r="X6" s="40"/>
-    </row>
-    <row r="7" spans="1:46" ht="30.75">
-      <c r="A7" s="46" t="s">
+      <c r="D6" s="4"/>
+      <c r="O6" s="32"/>
+      <c r="P6" s="32"/>
+      <c r="X6" s="34"/>
+    </row>
+    <row r="7" spans="1:46" ht="30" x14ac:dyDescent="0.25">
+      <c r="A7" s="38" t="s">
         <v>26</v>
       </c>
-      <c r="B7" s="47" t="s">
-        <v>3</v>
-      </c>
-      <c r="C7" s="47" t="s">
-        <v>3</v>
-      </c>
-      <c r="D7" s="5"/>
-      <c r="K7" s="38"/>
-      <c r="N7" s="38"/>
-      <c r="Q7" s="38"/>
-      <c r="AA7" s="38"/>
-    </row>
-    <row r="8" spans="1:46">
-      <c r="A8" s="48" t="s">
+      <c r="B7" s="39" t="s">
+        <v>3</v>
+      </c>
+      <c r="C7" s="39" t="s">
+        <v>3</v>
+      </c>
+      <c r="D7" s="4"/>
+      <c r="K7" s="32"/>
+      <c r="N7" s="32"/>
+      <c r="Q7" s="32"/>
+      <c r="AA7" s="32"/>
+    </row>
+    <row r="8" spans="1:46" x14ac:dyDescent="0.25">
+      <c r="A8" s="40" t="s">
         <v>17</v>
       </c>
-      <c r="B8" s="47" t="s">
-        <v>3</v>
-      </c>
-      <c r="C8" s="49">
+      <c r="B8" s="39" t="s">
+        <v>3</v>
+      </c>
+      <c r="C8" s="41">
         <v>26384888.600000001</v>
       </c>
-      <c r="D8" s="5"/>
-      <c r="E8" s="38"/>
-      <c r="F8" s="38"/>
-      <c r="G8" s="38"/>
-      <c r="H8" s="38"/>
-      <c r="I8" s="38"/>
-      <c r="J8" s="38"/>
-    </row>
-    <row r="9" spans="1:46">
-      <c r="A9" s="48" t="s">
+      <c r="D8" s="4"/>
+      <c r="E8" s="32"/>
+      <c r="F8" s="32"/>
+      <c r="G8" s="32"/>
+      <c r="H8" s="32"/>
+      <c r="I8" s="32"/>
+      <c r="J8" s="32"/>
+    </row>
+    <row r="9" spans="1:46" x14ac:dyDescent="0.25">
+      <c r="A9" s="40" t="s">
         <v>27</v>
       </c>
-      <c r="B9" s="47" t="s">
-        <v>3</v>
-      </c>
-      <c r="C9" s="49">
+      <c r="B9" s="39" t="s">
+        <v>3</v>
+      </c>
+      <c r="C9" s="41">
         <v>309363.3</v>
       </c>
-      <c r="D9" s="5"/>
-    </row>
-    <row r="10" spans="1:46">
-      <c r="A10" s="5"/>
-      <c r="B10" s="5"/>
-      <c r="C10" s="5"/>
-      <c r="D10" s="5"/>
-    </row>
-    <row r="11" spans="1:46">
-      <c r="A11" s="50" t="s">
+      <c r="D9" s="4"/>
+    </row>
+    <row r="10" spans="1:46" x14ac:dyDescent="0.25">
+      <c r="A10" s="4"/>
+      <c r="B10" s="4"/>
+      <c r="C10" s="4"/>
+      <c r="D10" s="4"/>
+    </row>
+    <row r="11" spans="1:46" x14ac:dyDescent="0.25">
+      <c r="A11" s="42" t="s">
         <v>28</v>
       </c>
-      <c r="B11" s="5"/>
-      <c r="C11" s="5"/>
-      <c r="D11" s="8" t="s">
+      <c r="B11" s="4"/>
+      <c r="C11" s="4"/>
+      <c r="D11" s="6" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="12" spans="1:46">
-      <c r="A12" s="5"/>
-      <c r="B12" s="5"/>
-      <c r="C12" s="5"/>
-      <c r="D12" s="5"/>
+    <row r="12" spans="1:46" x14ac:dyDescent="0.25">
+      <c r="A12" s="4"/>
+      <c r="B12" s="4"/>
+      <c r="C12" s="4"/>
+      <c r="D12" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1438,222 +1419,222 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DB5E8A3F-AE52-415F-9A67-4E8EEAC6AAFE}">
   <dimension ref="A1:D24"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="70.7109375" customWidth="1"/>
     <col min="2" max="2" width="14" customWidth="1"/>
     <col min="10" max="10" width="12.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4">
-      <c r="A1" s="5"/>
-      <c r="B1" s="5"/>
-      <c r="C1" s="5"/>
-    </row>
-    <row r="2" spans="1:4">
-      <c r="A2" s="5"/>
-      <c r="B2" s="5" t="s">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" s="4"/>
+      <c r="B1" s="4"/>
+      <c r="C1" s="4"/>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" s="4"/>
+      <c r="B2" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="C2" s="4" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="3" spans="1:4">
-      <c r="A3" s="14" t="s">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="B3" s="15">
+      <c r="B3" s="11">
         <f>13.9/100</f>
         <v>0.13900000000000001</v>
       </c>
-      <c r="C3" s="16" t="s">
+      <c r="C3" s="12" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:4">
-      <c r="A4" s="17" t="s">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" s="13" t="s">
         <v>32</v>
       </c>
-      <c r="B4" s="5">
+      <c r="B4" s="4">
         <f>1121064767261.88/10^6</f>
         <v>1121064.76726188</v>
       </c>
-      <c r="C4" s="10" t="s">
+      <c r="C4" s="8" t="s">
         <v>33</v>
       </c>
       <c r="D4" s="1"/>
     </row>
-    <row r="5" spans="1:4">
-      <c r="A5" s="17" t="s">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" s="13" t="s">
         <v>34</v>
       </c>
-      <c r="B5" s="19">
+      <c r="B5" s="15">
         <f>B4*B3</f>
         <v>155828.00264940134</v>
       </c>
-      <c r="C5" s="18" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4">
-      <c r="A6" s="17" t="s">
+      <c r="C5" s="14" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" s="13" t="s">
         <v>35</v>
       </c>
-      <c r="B6" s="20">
+      <c r="B6" s="16">
         <v>0.21</v>
       </c>
-      <c r="C6" s="10" t="s">
+      <c r="C6" s="8" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="7" spans="1:4">
-      <c r="A7" s="21" t="s">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" s="17" t="s">
         <v>36</v>
       </c>
-      <c r="B7" s="22">
+      <c r="B7" s="18">
         <f>B5*B6</f>
         <v>32723.880556374283</v>
       </c>
-      <c r="C7" s="23" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4">
-      <c r="A8" s="5"/>
-      <c r="B8" s="5"/>
-      <c r="C8" s="5"/>
-    </row>
-    <row r="9" spans="1:4">
-      <c r="A9" s="24"/>
-      <c r="B9" s="24"/>
-      <c r="C9" s="24"/>
-    </row>
-    <row r="10" spans="1:4">
-      <c r="A10" s="25" t="s">
+      <c r="C7" s="19" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" s="4"/>
+      <c r="B8" s="4"/>
+      <c r="C8" s="4"/>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" s="20"/>
+      <c r="B9" s="20"/>
+      <c r="C9" s="20"/>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" s="21" t="s">
         <v>37</v>
       </c>
-      <c r="B10" s="26">
+      <c r="B10" s="22">
         <f>B7*About!B29</f>
         <v>29029.703654250392</v>
       </c>
-      <c r="C10" s="27" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4">
-      <c r="A11" s="28" t="s">
-        <v>3</v>
-      </c>
-      <c r="B11" s="24"/>
-      <c r="C11" s="29" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4">
-      <c r="A12" s="28" t="s">
+      <c r="C10" s="23" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" s="24" t="s">
+        <v>3</v>
+      </c>
+      <c r="B11" s="20"/>
+      <c r="C11" s="25" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" s="24" t="s">
         <v>38</v>
       </c>
-      <c r="B12" s="30">
+      <c r="B12" s="26">
         <f>'Employee Compensation'!C9</f>
         <v>309363.3</v>
       </c>
-      <c r="C12" s="29" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4">
-      <c r="A13" s="28" t="s">
-        <v>3</v>
-      </c>
-      <c r="B13" s="24"/>
-      <c r="C13" s="29" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4">
-      <c r="A14" s="17" t="s">
-        <v>3</v>
-      </c>
-      <c r="B14" s="5"/>
-      <c r="C14" s="18" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4">
-      <c r="A15" s="28" t="s">
+      <c r="C12" s="25" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13" s="24" t="s">
+        <v>3</v>
+      </c>
+      <c r="B13" s="20"/>
+      <c r="C13" s="25" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="B14" s="4"/>
+      <c r="C14" s="14" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15" s="24" t="s">
         <v>39</v>
       </c>
-      <c r="B15" s="31">
+      <c r="B15" s="27">
         <f>B10/(B12)</f>
         <v>9.3836934291334467E-2</v>
       </c>
-      <c r="C15" s="29" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4">
-      <c r="A16" s="17" t="s">
-        <v>3</v>
-      </c>
-      <c r="B16" s="5"/>
-      <c r="C16" s="18" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3">
-      <c r="A17" s="28" t="s">
+      <c r="C15" s="25" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="B16" s="4"/>
+      <c r="C16" s="14" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17" s="24" t="s">
         <v>40</v>
       </c>
-      <c r="B17" s="5">
+      <c r="B17" s="4">
         <f>30/24</f>
         <v>1.25</v>
       </c>
-      <c r="C17" s="18" t="s">
+      <c r="C17" s="14" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="18" spans="1:3">
-      <c r="A18" s="32" t="s">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A18" s="28" t="s">
         <v>42</v>
       </c>
-      <c r="B18" s="33">
+      <c r="B18" s="29">
         <f>B15*B17</f>
         <v>0.11729616786416808</v>
       </c>
-      <c r="C18" s="23" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3">
-      <c r="A19" s="5"/>
-      <c r="B19" s="5"/>
-      <c r="C19" s="5"/>
-    </row>
-    <row r="20" spans="1:3">
-      <c r="A20" s="5"/>
-      <c r="B20" s="5"/>
-      <c r="C20" s="5"/>
-    </row>
-    <row r="21" spans="1:3">
-      <c r="A21" s="5"/>
-      <c r="B21" s="5"/>
-      <c r="C21" s="5"/>
-    </row>
-    <row r="22" spans="1:3">
-      <c r="A22" s="5"/>
-      <c r="B22" s="5"/>
-      <c r="C22" s="13"/>
-    </row>
-    <row r="23" spans="1:3">
-      <c r="A23" s="5"/>
-      <c r="B23" s="5"/>
-      <c r="C23" s="5"/>
-    </row>
-    <row r="24" spans="1:3">
-      <c r="A24" s="5"/>
-      <c r="B24" s="5"/>
-      <c r="C24" s="5"/>
+      <c r="C18" s="19" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A19" s="4"/>
+      <c r="B19" s="4"/>
+      <c r="C19" s="4"/>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A20" s="4"/>
+      <c r="B20" s="4"/>
+      <c r="C20" s="4"/>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A21" s="4"/>
+      <c r="B21" s="4"/>
+      <c r="C21" s="4"/>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A22" s="4"/>
+      <c r="B22" s="4"/>
+      <c r="C22" s="7"/>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A23" s="4"/>
+      <c r="B23" s="4"/>
+      <c r="C23" s="4"/>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A24" s="4"/>
+      <c r="B24" s="4"/>
+      <c r="C24" s="4"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -1671,21 +1652,21 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="26.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="28.5">
+    <row r="1" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="B1" s="2" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>44</v>
       </c>
-      <c r="B2" s="34">
+      <c r="B2" s="45">
         <f>Calculations!B18</f>
         <v>0.11729616786416808</v>
       </c>
@@ -1696,21 +1677,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101009A9DAB439B36DB4795F39C4E722C7BC4" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="44674c89fa9bc5e97a878a6680c46188">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="79748b23-d81a-423e-9112-21109dc864e6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="447839a363ea5a12024b5bf1ab53ed90" ns2:_="">
     <xsd:import namespace="79748b23-d81a-423e-9112-21109dc864e6"/>
@@ -1854,14 +1820,52 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C74E7ED2-25FB-471A-BC94-DE6A7944E36F}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3C90BB16-13A7-4F49-8AA0-ED926081FDA7}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="79748b23-d81a-423e-9112-21109dc864e6"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{416F06C2-C087-4F9D-8A20-363898D3F3B0}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{416F06C2-C087-4F9D-8A20-363898D3F3B0}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3C90BB16-13A7-4F49-8AA0-ED926081FDA7}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C74E7ED2-25FB-471A-BC94-DE6A7944E36F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>